<commit_message>
Publish Szeged_2024_WC, Samarkand_2024_WCH, Paris_2024_PG, Poznan_2024_WC
</commit_message>
<xml_diff>
--- a/events/Paris_2024_PG/Paris_2024_PG_Results.xlsx
+++ b/events/Paris_2024_PG/Paris_2024_PG_Results.xlsx
@@ -6606,6 +6606,11 @@
           <t>+1.40</t>
         </is>
       </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>98111</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -16917,6 +16922,11 @@
           <t>52.69</t>
         </is>
       </c>
+      <c r="R237" t="inlineStr">
+        <is>
+          <t>98111</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -20206,6 +20216,11 @@
       <c r="Q284" t="inlineStr">
         <is>
           <t>+1.34</t>
+        </is>
+      </c>
+      <c r="R284" t="inlineStr">
+        <is>
+          <t>98111</t>
         </is>
       </c>
     </row>
@@ -22277,7 +22292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D99"/>
+  <dimension ref="A1:D100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24458,6 +24473,28 @@
         </is>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>98111</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Steven</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>HAXTON</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>